<commit_message>
fix csv file names NBICP, RQSD, SoFCtMbCTPR, FOVTSTCT, ISFR
</commit_message>
<xml_diff>
--- a/InputData/ccs/NBICP/Non BAU Industry CCS Parameters.xlsx
+++ b/InputData/ccs/NBICP/Non BAU Industry CCS Parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ccs\NBICP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\ccs\NBICP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D4527F4-06B7-435E-8932-6A478272C4C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA685EF-7CC7-4227-AC0C-9EAE69FE1E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7770" yWindow="525" windowWidth="19110" windowHeight="16425" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Capacity Factor Data" sheetId="20" r:id="rId3"/>
     <sheet name="Current and Planned Capacity" sheetId="17" r:id="rId4"/>
     <sheet name="BAU Emissions" sheetId="21" r:id="rId5"/>
-    <sheet name="BBICP-CS" sheetId="22" r:id="rId6"/>
+    <sheet name="NBICP-CS" sheetId="22" r:id="rId6"/>
     <sheet name="NBICP-FoCPAbI-energyEmis" sheetId="18" r:id="rId7"/>
     <sheet name="NBICP-FoCPAbI-processEmis" sheetId="16" r:id="rId8"/>
   </sheets>

</xml_diff>